<commit_message>
Sync kobo folder with GPS and photo support
</commit_message>
<xml_diff>
--- a/kobo/YALL_MEAL_Indicator_Update.xlsx
+++ b/kobo/YALL_MEAL_Indicator_Update.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -716,17 +716,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Notes / context (optional)</t>
+          <t>GPS location (optional — tap to capture on site)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -743,22 +743,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>select_one coordinator</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>coordinator</t>
+          <t>photo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Recorded by</t>
+          <t>Photo evidence (optional)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -766,6 +766,60 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Notes / context (optional)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>select_one coordinator</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>coordinator</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Recorded by</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>